<commit_message>
Complete Raumbuch with VOB rules and corridor logic
</commit_message>
<xml_diff>
--- a/sample_data/raumbuch.xlsx
+++ b/sample_data/raumbuch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://thdegde-my.sharepoint.com/personal/amirhossein_farsinejad_th-deg_de/Documents/bimnexus/bim-nexus/sample_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_2B59D2BFD300D139D142DCF0501810F4560FF841" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF5C42C4-7BAC-487F-B8CB-938BB3268C67}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_2B59D2BFD390523ABDC1DFF05058F0347C8DE325" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD65E630-BA91-4257-98EB-830ECF1CC393}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
   <si>
     <t>Nr</t>
   </si>
@@ -43,7 +43,7 @@
     <t>Wand Brutto (m²)</t>
   </si>
   <si>
-    <t>Abzüge (m²)</t>
+    <t>Abzüge VOB (m²)</t>
   </si>
   <si>
     <t>Anstrich (m²)</t>
@@ -58,16 +58,22 @@
     <t>Decke (m²)</t>
   </si>
   <si>
-    <t>Türen</t>
-  </si>
-  <si>
-    <t>Fenster</t>
-  </si>
-  <si>
-    <t>Möbel</t>
-  </si>
-  <si>
-    <t>Ausstattung</t>
+    <t>Türen Anz.</t>
+  </si>
+  <si>
+    <t>Türen Details</t>
+  </si>
+  <si>
+    <t>Fenster Anz.</t>
+  </si>
+  <si>
+    <t>Fenster Details</t>
+  </si>
+  <si>
+    <t>Möbel Anz.</t>
+  </si>
+  <si>
+    <t>Möbel Details</t>
   </si>
   <si>
     <t>1</t>
@@ -79,6 +85,12 @@
     <t>EG</t>
   </si>
   <si>
+    <t xml:space="preserve"> x 2135:2435715 (0.89×2.31m=2.06m² [Abzug])</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> x 1400:2435823 (1.1×2.25m=2.48m²)</t>
+  </si>
+  <si>
     <t>Bett-01:1800 x 2000:2439864</t>
   </si>
   <si>
@@ -88,6 +100,12 @@
     <t>Livingroom</t>
   </si>
   <si>
+    <t xml:space="preserve"> x 2135:2435715 (0.89×2.31m=2.06m² [Korridor]),  x 2135:2435746 (0.88×2.31m=2.03m² [Abzug]),  x 2135:2436308 (0.88×2.31m=2.03m² [Korridor]),  x 2135:2436396 (0.88×2.31m=2.03m² [Korridor])</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> x 1400:2435864 (1.1×2.25m=2.48m²),  x 1400:2435977 (2.28×2.25m=5.13m²),  x 1400:2440802 (2.28×2.25m=5.13m²)</t>
+  </si>
+  <si>
     <t>Sofa-03:B 2000:2440064, Sofa-03:B 2000:2440280, Sofa-03:B 2000:2440370</t>
   </si>
   <si>
@@ -97,6 +115,9 @@
     <t>Kitchen</t>
   </si>
   <si>
+    <t xml:space="preserve"> x 1400:2435901 (1.1×2.25m=2.48m²)</t>
+  </si>
+  <si>
     <t>Küchenzeile-01 Generisch:Typ1:2436530, Küchenzeile-01 Generisch:Typ1:2437091, Küchenzeile-01 Generisch:Typ1:2437254</t>
   </si>
   <si>
@@ -106,10 +127,16 @@
     <t>Bathroom</t>
   </si>
   <si>
+    <t xml:space="preserve"> x 2135:2436308 (0.88×2.31m=2.03m² [Abzug])</t>
+  </si>
+  <si>
     <t>5</t>
   </si>
   <si>
     <t>WC</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> x 2135:2436396 (0.88×2.31m=2.03m² [Abzug])</t>
   </si>
 </sst>
 </file>
@@ -449,16 +476,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -507,16 +531,22 @@
       <c r="P1" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D2">
         <v>31.58</v>
@@ -548,25 +578,31 @@
       <c r="M2">
         <v>1</v>
       </c>
-      <c r="N2">
-        <v>1</v>
+      <c r="N2" t="s">
+        <v>21</v>
       </c>
       <c r="O2">
         <v>1</v>
       </c>
       <c r="P2" t="s">
-        <v>19</v>
+        <v>22</v>
+      </c>
+      <c r="Q2">
+        <v>1</v>
+      </c>
+      <c r="R2" t="s">
+        <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
         <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" t="s">
-        <v>18</v>
       </c>
       <c r="D3">
         <v>69.239999999999995</v>
@@ -581,10 +617,10 @@
         <v>81.400000000000006</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>10.26</v>
       </c>
       <c r="I3">
-        <v>81.400000000000006</v>
+        <v>71.14</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -598,25 +634,31 @@
       <c r="M3">
         <v>4</v>
       </c>
-      <c r="N3">
-        <v>3</v>
+      <c r="N3" t="s">
+        <v>26</v>
       </c>
       <c r="O3">
         <v>3</v>
       </c>
       <c r="P3" t="s">
-        <v>22</v>
+        <v>27</v>
+      </c>
+      <c r="Q3">
+        <v>3</v>
+      </c>
+      <c r="R3" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D4">
         <v>9.1999999999999993</v>
@@ -648,25 +690,28 @@
       <c r="M4">
         <v>0</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>1</v>
       </c>
-      <c r="O4">
+      <c r="P4" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q4">
         <v>3</v>
       </c>
-      <c r="P4" t="s">
-        <v>25</v>
+      <c r="R4" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D5">
         <v>5.59</v>
@@ -698,22 +743,25 @@
       <c r="M5">
         <v>1</v>
       </c>
-      <c r="N5">
-        <v>0</v>
+      <c r="N5" t="s">
+        <v>35</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D6">
         <v>6.83</v>
@@ -745,10 +793,13 @@
       <c r="M6">
         <v>1</v>
       </c>
-      <c r="N6">
-        <v>0</v>
+      <c r="N6" t="s">
+        <v>38</v>
       </c>
       <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
         <v>0</v>
       </c>
     </row>

</xml_diff>